<commit_message>
duy tinh tien loi co yen thang 02.2026
</commit_message>
<xml_diff>
--- a/ThuChiCoYenLinhTrung.xlsx
+++ b/ThuChiCoYenLinhTrung.xlsx
@@ -1,20 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" mc:Ignorable="x15">
-  <fileVersion appName="xl" lastEdited="6" lowestEdited="6" rupBuild="14420"/>
-  <workbookPr/>
-  <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
-    <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="G:\DUY-CLOUD\"/>
-    </mc:Choice>
-  </mc:AlternateContent>
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2">
+  <fileVersion appName="Calc"/>
+  <workbookPr backupFile="false" showObjects="all" date1904="false"/>
+  <workbookProtection/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="0" windowWidth="16380" windowHeight="8190" tabRatio="500"/>
+    <workbookView showHorizontalScroll="true" showVerticalScroll="true" showSheetTabs="true" xWindow="0" yWindow="0" windowWidth="16384" windowHeight="8192" tabRatio="500" firstSheet="0" activeTab="0"/>
   </bookViews>
   <sheets>
-    <sheet name="GhiNo" sheetId="1" r:id="rId1"/>
+    <sheet name="GhiNo" sheetId="1" state="visible" r:id="rId3"/>
   </sheets>
-  <calcPr calcId="152511" iterateDelta="1E-4"/>
+  <calcPr iterateCount="100" refMode="A1" iterate="false" iterateDelta="0.0001"/>
   <extLst>
     <ext xmlns:loext="http://schemas.libreoffice.org/" uri="{7626C862-2A13-11E5-B345-FEFF819CDC9F}">
       <loext:extCalcPr stringRefSyntax="ExcelA1"/>
@@ -24,349 +20,356 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="125" uniqueCount="112">
-  <si>
-    <t>500+1100+2700-105=</t>
-  </si>
-  <si>
-    <t>Cô Yến còn nợ trước đó</t>
-  </si>
-  <si>
-    <t>Còn lại từ  hóa đơn 10/05</t>
-  </si>
-  <si>
-    <t>Hóa đơn 29/06</t>
-  </si>
-  <si>
-    <t>Tiền xe tháng 06</t>
-  </si>
-  <si>
-    <t>10/07/2024</t>
-  </si>
-  <si>
-    <t>Tiền lãi tháng 06</t>
-  </si>
-  <si>
-    <t>16/07/2024</t>
-  </si>
-  <si>
-    <t>Hóa đơn 30/07</t>
-  </si>
-  <si>
-    <t>Tiền xe tháng 07</t>
-  </si>
-  <si>
-    <t>10/08/2024</t>
-  </si>
-  <si>
-    <t>Tiền lãi tháng 07</t>
-  </si>
-  <si>
-    <t>16/08/2024</t>
-  </si>
-  <si>
-    <t>Co Yến chuyển trả 3tr</t>
-  </si>
-  <si>
-    <t>17/08/2024</t>
-  </si>
-  <si>
-    <t>Tiền xe tháng 08</t>
-  </si>
-  <si>
-    <t>10/09/2024</t>
-  </si>
-  <si>
-    <t>Tiền lãi tháng 08</t>
-  </si>
-  <si>
-    <t>16/09/2024</t>
-  </si>
-  <si>
-    <t>Hóa đơn ngày 20/09</t>
-  </si>
-  <si>
-    <t>20/09/2024</t>
-  </si>
-  <si>
-    <t>Cô Yến chuyển khoản 1tr</t>
-  </si>
-  <si>
-    <t>23/09/2024</t>
-  </si>
-  <si>
-    <t>29/09/2024</t>
-  </si>
-  <si>
-    <t>Hóa đơn ngày 02/10</t>
-  </si>
-  <si>
-    <t>02/10/2024</t>
-  </si>
-  <si>
-    <t>Cô Yến chuyển 600k</t>
-  </si>
-  <si>
-    <t>04/10/2024</t>
-  </si>
-  <si>
-    <t>Cô Yến chuyển 400k</t>
-  </si>
-  <si>
-    <t>10/10/2024</t>
-  </si>
-  <si>
-    <t>Tiền xe tháng 09</t>
-  </si>
-  <si>
-    <t>Hóa đơn 14/10</t>
-  </si>
-  <si>
-    <t>14/10/2024</t>
-  </si>
-  <si>
-    <t>Tiền lãi tháng 10</t>
-  </si>
-  <si>
-    <t>16/10/2024</t>
-  </si>
-  <si>
-    <t>Cô Yến chuyển 2tr</t>
-  </si>
-  <si>
-    <t>21/10/2024</t>
-  </si>
-  <si>
-    <t>Hóa đơn ngày 29/10</t>
-  </si>
-  <si>
-    <t>29/10/2024</t>
-  </si>
-  <si>
-    <t>Cô Yến chuyển 1tr</t>
-  </si>
-  <si>
-    <t>Tiền xe tháng 10</t>
-  </si>
-  <si>
-    <t>10/11/2024</t>
-  </si>
-  <si>
-    <t>Hóa đơn ngày 12/11</t>
-  </si>
-  <si>
-    <t>12/11/2024</t>
-  </si>
-  <si>
-    <t>Tiền lãi tháng 11</t>
-  </si>
-  <si>
-    <t>16/11/2024</t>
-  </si>
-  <si>
-    <t>Hóa đơn ngày 26/11</t>
-  </si>
-  <si>
-    <t>26/11/2024</t>
-  </si>
-  <si>
-    <t>Hóa đơn ngày 10/12</t>
-  </si>
-  <si>
-    <t>10/12/2024</t>
-  </si>
-  <si>
-    <t>Cô Yến chuyển 3tr</t>
-  </si>
-  <si>
-    <t>11/12/2024</t>
-  </si>
-  <si>
-    <t>16/12/2024</t>
-  </si>
-  <si>
-    <t>Hóa đơn ngày 17/12</t>
-  </si>
-  <si>
-    <t>17/12/2024</t>
-  </si>
-  <si>
-    <t>Cô Yến chuyển trả 2tr</t>
-  </si>
-  <si>
-    <t>18/12/2024</t>
-  </si>
-  <si>
-    <t>Hóa đơn ngày 28/12</t>
-  </si>
-  <si>
-    <t>28/12/2024</t>
-  </si>
-  <si>
-    <t>29/12/2024</t>
-  </si>
-  <si>
-    <t>Hóa đơn ngày 08/01/2025</t>
-  </si>
-  <si>
-    <t>08/01/2025</t>
-  </si>
-  <si>
-    <t>09/01/2025</t>
-  </si>
-  <si>
-    <t>Lấy tiền lời cô Yến</t>
-  </si>
-  <si>
-    <t>16/01/2025</t>
-  </si>
-  <si>
-    <t>Hóa đơn ngày 16/01</t>
-  </si>
-  <si>
-    <t>Cô Yến chuyển 3tr</t>
-  </si>
-  <si>
-    <t>26/01/2025</t>
-  </si>
-  <si>
-    <t>hóa đơn ngày 04/02/2025</t>
-  </si>
-  <si>
-    <t>04/02/2025</t>
-  </si>
-  <si>
-    <t>Cô Yến chuyển 5tr</t>
-  </si>
-  <si>
-    <t>12/02/2025</t>
-  </si>
-  <si>
-    <t>Lấy tiền lời cô Yến tháng 01</t>
-  </si>
-  <si>
-    <t>16/02/2025</t>
-  </si>
-  <si>
-    <t>Hóa đơn ngày 18/02</t>
-  </si>
-  <si>
-    <t>18/02/2025</t>
-  </si>
-  <si>
-    <t>Lấy tiền lời cô Yến tháng 02</t>
-  </si>
-  <si>
-    <t>16/03/2025</t>
-  </si>
-  <si>
-    <t>Hóa đơn ngày 17/03</t>
-  </si>
-  <si>
-    <t>17/03/2025</t>
-  </si>
-  <si>
-    <t>Hóa đơn ngày 31/03</t>
-  </si>
-  <si>
-    <t>31/03/2025</t>
-  </si>
-  <si>
-    <t>Hóa đơn ngày 08/04/2025</t>
-  </si>
-  <si>
-    <t>08/04/2025</t>
-  </si>
-  <si>
-    <t>Cô Yến trả 3tr</t>
-  </si>
-  <si>
-    <t>Cô Yến trả 700k</t>
-  </si>
-  <si>
-    <t>10/04/2025</t>
-  </si>
-  <si>
-    <t>Lấy tiền lời cô Yến tháng 03</t>
-  </si>
-  <si>
-    <t>16/04/2025</t>
-  </si>
-  <si>
-    <t>Hóa đơn ngày 23/04</t>
-  </si>
-  <si>
-    <t>23/04/2025</t>
-  </si>
-  <si>
-    <t>Lấy tiền lời cô Yến tháng 04</t>
-  </si>
-  <si>
-    <t>16/05/2025</t>
-  </si>
-  <si>
-    <t>Chuyển cô Yến 4tr</t>
-  </si>
-  <si>
-    <t>22/05/2025</t>
-  </si>
-  <si>
-    <t>Lấy tiền lời cô Yến tháng 05</t>
-  </si>
-  <si>
-    <t>16/06/2025</t>
-  </si>
-  <si>
-    <t>Lấy tiền lời cô Yến tháng 06</t>
-  </si>
-  <si>
-    <t>16/07/2025</t>
-  </si>
-  <si>
-    <t>Lấy tiền lời cô Yến tháng 07</t>
-  </si>
-  <si>
-    <t>16/08/2025</t>
-  </si>
-  <si>
-    <t>Lấy tiền lời cô Yến tháng 08</t>
-  </si>
-  <si>
-    <t>16/09/2025</t>
-  </si>
-  <si>
-    <t>Lấy tiền lời cô Yến tháng 09</t>
-  </si>
-  <si>
-    <t>16/10/2025</t>
-  </si>
-  <si>
-    <t>Lấy tiền lời cô Yến tháng 10</t>
-  </si>
-  <si>
-    <t>16/11/2025</t>
-  </si>
-  <si>
-    <t>Lấy tiền lời cô Yến tháng 11</t>
-  </si>
-  <si>
-    <t>16/12/2025</t>
-  </si>
-  <si>
-    <t>Lấy tiền lời cô Yến tháng 12</t>
-  </si>
-  <si>
-    <t>Hiện tại</t>
-  </si>
-  <si>
-    <t>16/02/2026</t>
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="127" uniqueCount="113">
+  <si>
+    <t xml:space="preserve">500+1100+2700-105=</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Cô Yến còn nợ trước đó</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Còn lại từ  hóa đơn 10/05</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Hóa đơn 29/06</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Tiền xe tháng 06</t>
+  </si>
+  <si>
+    <t xml:space="preserve">10/07/2024</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Tiền lãi tháng 06</t>
+  </si>
+  <si>
+    <t xml:space="preserve">16/07/2024</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Hóa đơn 30/07</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Tiền xe tháng 07</t>
+  </si>
+  <si>
+    <t xml:space="preserve">10/08/2024</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Tiền lãi tháng 07</t>
+  </si>
+  <si>
+    <t xml:space="preserve">16/08/2024</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Co Yến chuyển trả 3tr</t>
+  </si>
+  <si>
+    <t xml:space="preserve">17/08/2024</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Tiền xe tháng 08</t>
+  </si>
+  <si>
+    <t xml:space="preserve">10/09/2024</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Tiền lãi tháng 08</t>
+  </si>
+  <si>
+    <t xml:space="preserve">16/09/2024</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Hóa đơn ngày 20/09</t>
+  </si>
+  <si>
+    <t xml:space="preserve">20/09/2024</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Cô Yến chuyển khoản 1tr</t>
+  </si>
+  <si>
+    <t xml:space="preserve">23/09/2024</t>
+  </si>
+  <si>
+    <t xml:space="preserve">29/09/2024</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Hóa đơn ngày 02/10</t>
+  </si>
+  <si>
+    <t xml:space="preserve">02/10/2024</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Cô Yến chuyển 600k</t>
+  </si>
+  <si>
+    <t xml:space="preserve">04/10/2024</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Cô Yến chuyển 400k</t>
+  </si>
+  <si>
+    <t xml:space="preserve">10/10/2024</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Tiền xe tháng 09</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Hóa đơn 14/10</t>
+  </si>
+  <si>
+    <t xml:space="preserve">14/10/2024</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Tiền lãi tháng 10</t>
+  </si>
+  <si>
+    <t xml:space="preserve">16/10/2024</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Cô Yến chuyển 2tr</t>
+  </si>
+  <si>
+    <t xml:space="preserve">21/10/2024</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Hóa đơn ngày 29/10</t>
+  </si>
+  <si>
+    <t xml:space="preserve">29/10/2024</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Cô Yến chuyển 1tr</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Tiền xe tháng 10</t>
+  </si>
+  <si>
+    <t xml:space="preserve">10/11/2024</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Hóa đơn ngày 12/11</t>
+  </si>
+  <si>
+    <t xml:space="preserve">12/11/2024</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Tiền lãi tháng 11</t>
+  </si>
+  <si>
+    <t xml:space="preserve">16/11/2024</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Hóa đơn ngày 26/11</t>
+  </si>
+  <si>
+    <t xml:space="preserve">26/11/2024</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Hóa đơn ngày 10/12</t>
+  </si>
+  <si>
+    <t xml:space="preserve">10/12/2024</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Cô Yến chuyển 3tr</t>
+  </si>
+  <si>
+    <t xml:space="preserve">11/12/2024</t>
+  </si>
+  <si>
+    <t xml:space="preserve">16/12/2024</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Hóa đơn ngày 17/12</t>
+  </si>
+  <si>
+    <t xml:space="preserve">17/12/2024</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Cô Yến chuyển trả 2tr</t>
+  </si>
+  <si>
+    <t xml:space="preserve">18/12/2024</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Hóa đơn ngày 28/12</t>
+  </si>
+  <si>
+    <t xml:space="preserve">28/12/2024</t>
+  </si>
+  <si>
+    <t xml:space="preserve">29/12/2024</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Hóa đơn ngày 08/01/2025</t>
+  </si>
+  <si>
+    <t xml:space="preserve">08/01/2025</t>
+  </si>
+  <si>
+    <t xml:space="preserve">09/01/2025</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Lấy tiền lời cô Yến</t>
+  </si>
+  <si>
+    <t xml:space="preserve">16/01/2025</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Hóa đơn ngày 16/01</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Cô Yến chuyển 3tr</t>
+  </si>
+  <si>
+    <t xml:space="preserve">26/01/2025</t>
+  </si>
+  <si>
+    <t xml:space="preserve">hóa đơn ngày 04/02/2025</t>
+  </si>
+  <si>
+    <t xml:space="preserve">04/02/2025</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Cô Yến chuyển 5tr</t>
+  </si>
+  <si>
+    <t xml:space="preserve">12/02/2025</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Lấy tiền lời cô Yến tháng 01</t>
+  </si>
+  <si>
+    <t xml:space="preserve">16/02/2025</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Hóa đơn ngày 18/02</t>
+  </si>
+  <si>
+    <t xml:space="preserve">18/02/2025</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Lấy tiền lời cô Yến tháng 02</t>
+  </si>
+  <si>
+    <t xml:space="preserve">16/03/2025</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Hóa đơn ngày 17/03</t>
+  </si>
+  <si>
+    <t xml:space="preserve">17/03/2025</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Hóa đơn ngày 31/03</t>
+  </si>
+  <si>
+    <t xml:space="preserve">31/03/2025</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Hóa đơn ngày 08/04/2025</t>
+  </si>
+  <si>
+    <t xml:space="preserve">08/04/2025</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Cô Yến trả 3tr</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Cô Yến trả 700k</t>
+  </si>
+  <si>
+    <t xml:space="preserve">10/04/2025</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Lấy tiền lời cô Yến tháng 03</t>
+  </si>
+  <si>
+    <t xml:space="preserve">16/04/2025</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Hóa đơn ngày 23/04</t>
+  </si>
+  <si>
+    <t xml:space="preserve">23/04/2025</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Lấy tiền lời cô Yến tháng 04</t>
+  </si>
+  <si>
+    <t xml:space="preserve">16/05/2025</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Chuyển cô Yến 4tr</t>
+  </si>
+  <si>
+    <t xml:space="preserve">22/05/2025</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Lấy tiền lời cô Yến tháng 05</t>
+  </si>
+  <si>
+    <t xml:space="preserve">16/06/2025</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Lấy tiền lời cô Yến tháng 06</t>
+  </si>
+  <si>
+    <t xml:space="preserve">16/07/2025</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Lấy tiền lời cô Yến tháng 07</t>
+  </si>
+  <si>
+    <t xml:space="preserve">16/08/2025</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Lấy tiền lời cô Yến tháng 08</t>
+  </si>
+  <si>
+    <t xml:space="preserve">16/09/2025</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Lấy tiền lời cô Yến tháng 09</t>
+  </si>
+  <si>
+    <t xml:space="preserve">16/10/2025</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Lấy tiền lời cô Yến tháng 10</t>
+  </si>
+  <si>
+    <t xml:space="preserve">16/11/2025</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Lấy tiền lời cô Yến tháng 11</t>
+  </si>
+  <si>
+    <t xml:space="preserve">16/12/2025</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Lấy tiền lời cô Yến tháng 12</t>
+  </si>
+  <si>
+    <t xml:space="preserve">16/02/2026</t>
+  </si>
+  <si>
+    <t xml:space="preserve">16/03/2026</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Hiện tại</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <fonts count="3" x14ac:knownFonts="1">
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <numFmts count="2">
+    <numFmt numFmtId="164" formatCode="General"/>
+    <numFmt numFmtId="165" formatCode="@"/>
+  </numFmts>
+  <fonts count="6">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -375,7 +378,22 @@
       <charset val="1"/>
     </font>
     <font>
-      <b/>
+      <sz val="10"/>
+      <name val="Arial"/>
+      <family val="0"/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <name val="Arial"/>
+      <family val="0"/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <name val="Arial"/>
+      <family val="0"/>
+    </font>
+    <font>
+      <b val="true"/>
       <sz val="14"/>
       <color theme="1"/>
       <name val="Calibri"/>
@@ -383,7 +401,7 @@
       <charset val="1"/>
     </font>
     <font>
-      <b/>
+      <b val="true"/>
       <sz val="16"/>
       <color theme="1"/>
       <name val="Calibri"/>
@@ -406,7 +424,7 @@
     </fill>
   </fills>
   <borders count="1">
-    <border>
+    <border diagonalUp="false" diagonalDown="false">
       <left/>
       <right/>
       <top/>
@@ -414,27 +432,69 @@
       <diagonal/>
     </border>
   </borders>
-  <cellStyleXfs count="1">
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
+  <cellStyleXfs count="20">
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
+    <xf numFmtId="43" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
+    <xf numFmtId="41" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
+    <xf numFmtId="44" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
+    <xf numFmtId="42" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
+    <xf numFmtId="9" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
   </cellStyleXfs>
   <cellXfs count="7">
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
-      <alignment horizontal="center"/>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="false" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="49" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
-    <xf numFmtId="49" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
-      <alignment horizontal="right"/>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="49" fontId="1" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="165" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="false" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="165" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="right" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="165" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="4" fillId="2" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
   </cellXfs>
-  <cellStyles count="1">
+  <cellStyles count="6">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
+    <cellStyle name="Comma" xfId="15" builtinId="3"/>
+    <cellStyle name="Comma [0]" xfId="16" builtinId="6"/>
+    <cellStyle name="Currency" xfId="17" builtinId="4"/>
+    <cellStyle name="Currency [0]" xfId="18" builtinId="7"/>
+    <cellStyle name="Percent" xfId="19" builtinId="5"/>
   </cellStyles>
-  <dxfs count="0"/>
-  <tableStyles count="0" defaultTableStyle="TableStyleMedium2" defaultPivotStyle="PivotStyleLight16"/>
   <colors>
     <indexedColors>
       <rgbColor rgb="FF000000"/>
@@ -493,63 +553,47 @@
       <rgbColor rgb="FF993366"/>
       <rgbColor rgb="FF333399"/>
       <rgbColor rgb="FF333333"/>
-      <rgbColor rgb="00003366"/>
-      <rgbColor rgb="00339966"/>
-      <rgbColor rgb="00003300"/>
-      <rgbColor rgb="00333300"/>
-      <rgbColor rgb="00993300"/>
-      <rgbColor rgb="00993366"/>
-      <rgbColor rgb="00333399"/>
-      <rgbColor rgb="00333333"/>
     </indexedColors>
   </colors>
-  <extLst>
-    <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{EB79DEF2-80B8-43e5-95BD-54CBDDF9020C}">
-      <x14:slicerStyles defaultSlicerStyle="SlicerStyleLight1"/>
-    </ext>
-    <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{9260A510-F301-46a8-8635-F512D64BE5F5}">
-      <x15:timelineStyles defaultTimelineStyle="TimeSlicerStyleLight1"/>
-    </ext>
-  </extLst>
 </styleSheet>
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
-<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office Theme">
+<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Office Theme">
   <a:themeElements>
     <a:clrScheme name="Office">
       <a:dk1>
         <a:srgbClr val="000000"/>
       </a:dk1>
       <a:lt1>
-        <a:srgbClr val="FFFFFF"/>
+        <a:srgbClr val="ffffff"/>
       </a:lt1>
       <a:dk2>
-        <a:srgbClr val="1F497D"/>
+        <a:srgbClr val="1f497d"/>
       </a:dk2>
       <a:lt2>
-        <a:srgbClr val="EEECE1"/>
+        <a:srgbClr val="eeece1"/>
       </a:lt2>
       <a:accent1>
-        <a:srgbClr val="4F81BD"/>
+        <a:srgbClr val="4f81bd"/>
       </a:accent1>
       <a:accent2>
-        <a:srgbClr val="C0504D"/>
+        <a:srgbClr val="c0504d"/>
       </a:accent2>
       <a:accent3>
-        <a:srgbClr val="9BBB59"/>
+        <a:srgbClr val="9bbb59"/>
       </a:accent3>
       <a:accent4>
-        <a:srgbClr val="8064A2"/>
+        <a:srgbClr val="8064a2"/>
       </a:accent4>
       <a:accent5>
-        <a:srgbClr val="4BACC6"/>
+        <a:srgbClr val="4bacc6"/>
       </a:accent5>
       <a:accent6>
-        <a:srgbClr val="F79646"/>
+        <a:srgbClr val="f79646"/>
       </a:accent6>
       <a:hlink>
-        <a:srgbClr val="0000FF"/>
+        <a:srgbClr val="0000ff"/>
       </a:hlink>
       <a:folHlink>
         <a:srgbClr val="800080"/>
@@ -557,12 +601,12 @@
     </a:clrScheme>
     <a:fontScheme name="Office">
       <a:majorFont>
-        <a:latin typeface="Cambria" panose="020F0302020204030204"/>
+        <a:latin typeface="Cambria" panose="020F0302020204030204" pitchFamily="0" charset="1"/>
         <a:ea typeface=""/>
         <a:cs typeface=""/>
       </a:majorFont>
       <a:minorFont>
-        <a:latin typeface="Calibri" panose="020F0502020204030204"/>
+        <a:latin typeface="Calibri" panose="020F0502020204030204" pitchFamily="0" charset="1"/>
         <a:ea typeface=""/>
         <a:cs typeface=""/>
       </a:minorFont>
@@ -591,7 +635,7 @@
             </a:gs>
           </a:gsLst>
           <a:lin ang="16200000" scaled="1"/>
-          <a:tileRect/>
+          <a:tileRect l="0" t="0" r="0" b="0"/>
         </a:gradFill>
         <a:gradFill>
           <a:gsLst>
@@ -612,7 +656,7 @@
             </a:gs>
           </a:gsLst>
           <a:lin ang="16200000" scaled="0"/>
-          <a:tileRect/>
+          <a:tileRect l="0" t="0" r="0" b="0"/>
         </a:gradFill>
       </a:fillStyleLst>
       <a:lnStyleLst>
@@ -663,7 +707,7 @@
           <a:path path="circle">
             <a:fillToRect l="50000" t="-80000" r="50000" b="180000"/>
           </a:path>
-          <a:tileRect/>
+          <a:tileRect l="0" t="0" r="0" b="0"/>
         </a:gradFill>
         <a:gradFill>
           <a:gsLst>
@@ -681,738 +725,757 @@
           <a:path path="circle">
             <a:fillToRect l="50000" t="50000" r="50000" b="50000"/>
           </a:path>
-          <a:tileRect/>
+          <a:tileRect l="0" t="0" r="0" b="0"/>
         </a:gradFill>
       </a:bgFillStyleLst>
     </a:fmtScheme>
   </a:themeElements>
-  <a:objectDefaults/>
-  <a:extraClrSchemeLst/>
 </a:theme>
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A2:D151"/>
-  <sheetFormatPr defaultColWidth="8.7109375" defaultRowHeight="15" customHeight="1" x14ac:dyDescent="0.25"/>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+  <sheetPr filterMode="false">
+    <pageSetUpPr fitToPage="false"/>
+  </sheetPr>
+  <dimension ref="A2:D154"/>
+  <sheetFormatPr defaultColWidth="8.71484375" defaultRowHeight="15" customHeight="true" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
-    <col min="1" max="1" width="25.28515625" style="1" customWidth="1"/>
-    <col min="2" max="2" width="30.140625" style="2" customWidth="1"/>
-    <col min="3" max="3" width="17.85546875" customWidth="1"/>
-    <col min="4" max="4" width="17.42578125" style="3" customWidth="1"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="1" width="25.29"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="2" width="30.14"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="0" width="17.86"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="4" style="3" width="17.42"/>
   </cols>
   <sheetData>
-    <row r="2" spans="2:4" x14ac:dyDescent="0.25">
+    <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B2" s="2" t="s">
         <v>0</v>
       </c>
-      <c r="C2">
-        <f>500+1100+2700-105</f>
+      <c r="C2" s="0" t="n">
+        <f aca="false">500+1100+2700-105</f>
         <v>4195</v>
       </c>
     </row>
-    <row r="9" spans="2:4" x14ac:dyDescent="0.25">
+    <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B9" s="2" t="s">
         <v>1</v>
       </c>
-      <c r="C9">
+      <c r="C9" s="0" t="n">
         <v>195</v>
       </c>
     </row>
-    <row r="10" spans="2:4" x14ac:dyDescent="0.25">
+    <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B10" s="2" t="s">
         <v>2</v>
       </c>
-      <c r="C10">
+      <c r="C10" s="0" t="n">
         <v>1836</v>
       </c>
     </row>
-    <row r="11" spans="2:4" x14ac:dyDescent="0.25">
+    <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B11" s="2" t="s">
         <v>3</v>
       </c>
-      <c r="C11">
+      <c r="C11" s="0" t="n">
         <v>2540</v>
       </c>
     </row>
-    <row r="12" spans="2:4" x14ac:dyDescent="0.25">
+    <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B12" s="2" t="s">
         <v>4</v>
       </c>
-      <c r="C12">
+      <c r="C12" s="0" t="n">
         <v>1500</v>
       </c>
       <c r="D12" s="3" t="s">
         <v>5</v>
       </c>
     </row>
-    <row r="13" spans="2:4" x14ac:dyDescent="0.25">
+    <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B13" s="2" t="s">
         <v>6</v>
       </c>
-      <c r="C13">
+      <c r="C13" s="0" t="n">
         <v>3000</v>
       </c>
       <c r="D13" s="3" t="s">
         <v>7</v>
       </c>
     </row>
-    <row r="14" spans="2:4" x14ac:dyDescent="0.25">
+    <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B14" s="2" t="s">
         <v>8</v>
       </c>
-      <c r="C14">
+      <c r="C14" s="0" t="n">
         <v>2954</v>
       </c>
     </row>
-    <row r="15" spans="2:4" x14ac:dyDescent="0.25">
+    <row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B15" s="2" t="s">
         <v>9</v>
       </c>
-      <c r="C15">
+      <c r="C15" s="0" t="n">
         <v>1500</v>
       </c>
       <c r="D15" s="3" t="s">
         <v>10</v>
       </c>
     </row>
-    <row r="16" spans="2:4" x14ac:dyDescent="0.25">
+    <row r="16" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B16" s="2" t="s">
         <v>11</v>
       </c>
-      <c r="C16">
+      <c r="C16" s="0" t="n">
         <v>3000</v>
       </c>
       <c r="D16" s="3" t="s">
         <v>12</v>
       </c>
     </row>
-    <row r="17" spans="2:4" x14ac:dyDescent="0.25">
+    <row r="17" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B17" s="2" t="s">
         <v>13</v>
       </c>
-      <c r="C17">
+      <c r="C17" s="0" t="n">
         <v>-3000</v>
       </c>
       <c r="D17" s="3" t="s">
         <v>14</v>
       </c>
     </row>
-    <row r="18" spans="2:4" x14ac:dyDescent="0.25">
+    <row r="18" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B18" s="2" t="s">
         <v>15</v>
       </c>
-      <c r="C18">
+      <c r="C18" s="0" t="n">
         <v>1500</v>
       </c>
       <c r="D18" s="3" t="s">
         <v>16</v>
       </c>
     </row>
-    <row r="19" spans="2:4" x14ac:dyDescent="0.25">
+    <row r="19" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B19" s="2" t="s">
         <v>17</v>
       </c>
-      <c r="C19">
+      <c r="C19" s="0" t="n">
         <v>3000</v>
       </c>
       <c r="D19" s="3" t="s">
         <v>18</v>
       </c>
     </row>
-    <row r="20" spans="2:4" x14ac:dyDescent="0.25">
+    <row r="20" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B20" s="2" t="s">
         <v>19</v>
       </c>
-      <c r="C20">
+      <c r="C20" s="0" t="n">
         <v>1460</v>
       </c>
       <c r="D20" s="3" t="s">
         <v>20</v>
       </c>
     </row>
-    <row r="21" spans="2:4" x14ac:dyDescent="0.25">
+    <row r="21" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B21" s="2" t="s">
         <v>21</v>
       </c>
-      <c r="C21">
+      <c r="C21" s="0" t="n">
         <v>-1000</v>
       </c>
       <c r="D21" s="3" t="s">
         <v>22</v>
       </c>
     </row>
-    <row r="22" spans="2:4" x14ac:dyDescent="0.25">
+    <row r="22" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B22" s="2" t="s">
         <v>21</v>
       </c>
-      <c r="C22">
+      <c r="C22" s="0" t="n">
         <v>-1000</v>
       </c>
       <c r="D22" s="3" t="s">
         <v>23</v>
       </c>
     </row>
-    <row r="23" spans="2:4" x14ac:dyDescent="0.25">
+    <row r="23" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B23" s="2" t="s">
         <v>24</v>
       </c>
-      <c r="C23">
+      <c r="C23" s="0" t="n">
         <v>1350</v>
       </c>
       <c r="D23" s="3" t="s">
         <v>25</v>
       </c>
     </row>
-    <row r="24" spans="2:4" x14ac:dyDescent="0.25">
+    <row r="24" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B24" s="2" t="s">
         <v>26</v>
       </c>
-      <c r="C24">
+      <c r="C24" s="0" t="n">
         <v>-600</v>
       </c>
       <c r="D24" s="3" t="s">
         <v>27</v>
       </c>
     </row>
-    <row r="25" spans="2:4" x14ac:dyDescent="0.25">
+    <row r="25" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B25" s="2" t="s">
         <v>28</v>
       </c>
-      <c r="C25">
+      <c r="C25" s="0" t="n">
         <v>-400</v>
       </c>
       <c r="D25" s="3" t="s">
         <v>29</v>
       </c>
     </row>
-    <row r="26" spans="2:4" x14ac:dyDescent="0.25">
+    <row r="26" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B26" s="2" t="s">
         <v>30</v>
       </c>
-      <c r="C26">
+      <c r="C26" s="0" t="n">
         <v>1500</v>
       </c>
       <c r="D26" s="3" t="s">
         <v>29</v>
       </c>
     </row>
-    <row r="27" spans="2:4" x14ac:dyDescent="0.25">
+    <row r="27" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B27" s="2" t="s">
         <v>31</v>
       </c>
-      <c r="C27">
+      <c r="C27" s="0" t="n">
         <v>3200</v>
       </c>
       <c r="D27" s="3" t="s">
         <v>32</v>
       </c>
     </row>
-    <row r="28" spans="2:4" x14ac:dyDescent="0.25">
+    <row r="28" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B28" s="2" t="s">
         <v>33</v>
       </c>
-      <c r="C28">
+      <c r="C28" s="0" t="n">
         <v>3000</v>
       </c>
       <c r="D28" s="3" t="s">
         <v>34</v>
       </c>
     </row>
-    <row r="29" spans="2:4" x14ac:dyDescent="0.25">
+    <row r="29" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B29" s="2" t="s">
         <v>35</v>
       </c>
-      <c r="C29">
+      <c r="C29" s="0" t="n">
         <v>-2000</v>
       </c>
       <c r="D29" s="3" t="s">
         <v>36</v>
       </c>
     </row>
-    <row r="30" spans="2:4" x14ac:dyDescent="0.25">
+    <row r="30" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B30" s="2" t="s">
         <v>37</v>
       </c>
-      <c r="C30">
+      <c r="C30" s="0" t="n">
         <v>1730</v>
       </c>
       <c r="D30" s="3" t="s">
         <v>38</v>
       </c>
     </row>
-    <row r="31" spans="2:4" x14ac:dyDescent="0.25">
+    <row r="31" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B31" s="2" t="s">
         <v>39</v>
       </c>
-      <c r="C31">
+      <c r="C31" s="0" t="n">
         <v>-1000</v>
       </c>
       <c r="D31" s="3" t="s">
         <v>38</v>
       </c>
     </row>
-    <row r="32" spans="2:4" x14ac:dyDescent="0.25">
+    <row r="32" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B32" s="2" t="s">
         <v>40</v>
       </c>
-      <c r="C32">
+      <c r="C32" s="0" t="n">
         <v>1500</v>
       </c>
       <c r="D32" s="3" t="s">
         <v>41</v>
       </c>
     </row>
-    <row r="33" spans="2:4" x14ac:dyDescent="0.25">
+    <row r="33" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B33" s="2" t="s">
         <v>42</v>
       </c>
-      <c r="C33">
+      <c r="C33" s="0" t="n">
         <v>2000</v>
       </c>
       <c r="D33" s="3" t="s">
         <v>43</v>
       </c>
     </row>
-    <row r="34" spans="2:4" x14ac:dyDescent="0.25">
+    <row r="34" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B34" s="2" t="s">
         <v>44</v>
       </c>
-      <c r="C34">
+      <c r="C34" s="0" t="n">
         <v>3000</v>
       </c>
       <c r="D34" s="3" t="s">
         <v>45</v>
       </c>
     </row>
-    <row r="35" spans="2:4" x14ac:dyDescent="0.25">
+    <row r="35" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B35" s="2" t="s">
         <v>46</v>
       </c>
-      <c r="C35">
+      <c r="C35" s="0" t="n">
         <v>2000</v>
       </c>
       <c r="D35" s="3" t="s">
         <v>47</v>
       </c>
     </row>
-    <row r="36" spans="2:4" x14ac:dyDescent="0.25">
+    <row r="36" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B36" s="2" t="s">
         <v>48</v>
       </c>
-      <c r="C36">
+      <c r="C36" s="0" t="n">
         <v>2930</v>
       </c>
       <c r="D36" s="3" t="s">
         <v>49</v>
       </c>
     </row>
-    <row r="37" spans="2:4" x14ac:dyDescent="0.25">
+    <row r="37" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B37" s="2" t="s">
         <v>50</v>
       </c>
-      <c r="C37">
+      <c r="C37" s="0" t="n">
         <v>-3000</v>
       </c>
       <c r="D37" s="3" t="s">
         <v>51</v>
       </c>
     </row>
-    <row r="38" spans="2:4" x14ac:dyDescent="0.25">
+    <row r="38" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B38" s="2" t="s">
         <v>44</v>
       </c>
-      <c r="C38">
+      <c r="C38" s="0" t="n">
         <v>3000</v>
       </c>
       <c r="D38" s="3" t="s">
         <v>52</v>
       </c>
     </row>
-    <row r="39" spans="2:4" x14ac:dyDescent="0.25">
+    <row r="39" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B39" s="2" t="s">
         <v>53</v>
       </c>
-      <c r="C39">
+      <c r="C39" s="0" t="n">
         <v>1730</v>
       </c>
       <c r="D39" s="3" t="s">
         <v>54</v>
       </c>
     </row>
-    <row r="40" spans="2:4" x14ac:dyDescent="0.25">
+    <row r="40" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B40" s="2" t="s">
         <v>55</v>
       </c>
-      <c r="C40">
+      <c r="C40" s="0" t="n">
         <v>-2000</v>
       </c>
       <c r="D40" s="3" t="s">
         <v>56</v>
       </c>
     </row>
-    <row r="41" spans="2:4" x14ac:dyDescent="0.25">
+    <row r="41" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B41" s="2" t="s">
         <v>57</v>
       </c>
-      <c r="C41">
+      <c r="C41" s="0" t="n">
         <v>1920</v>
       </c>
       <c r="D41" s="3" t="s">
         <v>58</v>
       </c>
     </row>
-    <row r="42" spans="2:4" x14ac:dyDescent="0.25">
+    <row r="42" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B42" s="2" t="s">
         <v>35</v>
       </c>
-      <c r="C42">
+      <c r="C42" s="0" t="n">
         <v>-2000</v>
       </c>
       <c r="D42" s="3" t="s">
         <v>59</v>
       </c>
     </row>
-    <row r="43" spans="2:4" x14ac:dyDescent="0.25">
+    <row r="43" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B43" s="2" t="s">
         <v>60</v>
       </c>
-      <c r="C43">
+      <c r="C43" s="0" t="n">
         <v>1730</v>
       </c>
       <c r="D43" s="3" t="s">
         <v>61</v>
       </c>
     </row>
-    <row r="44" spans="2:4" x14ac:dyDescent="0.25">
+    <row r="44" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B44" s="2" t="s">
         <v>35</v>
       </c>
-      <c r="C44">
+      <c r="C44" s="0" t="n">
         <v>-2000</v>
       </c>
       <c r="D44" s="3" t="s">
         <v>62</v>
       </c>
     </row>
-    <row r="45" spans="2:4" x14ac:dyDescent="0.25">
+    <row r="45" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B45" s="2" t="s">
         <v>63</v>
       </c>
-      <c r="C45">
+      <c r="C45" s="0" t="n">
         <v>3000</v>
       </c>
       <c r="D45" s="3" t="s">
         <v>64</v>
       </c>
     </row>
-    <row r="46" spans="2:4" x14ac:dyDescent="0.25">
+    <row r="46" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B46" s="2" t="s">
         <v>65</v>
       </c>
-      <c r="C46">
+      <c r="C46" s="0" t="n">
         <v>810</v>
       </c>
       <c r="D46" s="3" t="s">
         <v>64</v>
       </c>
     </row>
-    <row r="47" spans="2:4" x14ac:dyDescent="0.25">
+    <row r="47" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B47" s="2" t="s">
         <v>66</v>
       </c>
-      <c r="C47">
+      <c r="C47" s="0" t="n">
         <v>-3000</v>
       </c>
       <c r="D47" s="3" t="s">
         <v>67</v>
       </c>
     </row>
-    <row r="48" spans="2:4" x14ac:dyDescent="0.25">
+    <row r="48" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B48" s="2" t="s">
         <v>68</v>
       </c>
-      <c r="C48">
+      <c r="C48" s="0" t="n">
         <v>3430</v>
       </c>
       <c r="D48" s="3" t="s">
         <v>69</v>
       </c>
     </row>
-    <row r="49" spans="2:4" x14ac:dyDescent="0.25">
+    <row r="49" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B49" s="2" t="s">
         <v>70</v>
       </c>
-      <c r="C49">
+      <c r="C49" s="0" t="n">
         <v>-5000</v>
       </c>
       <c r="D49" s="3" t="s">
         <v>71</v>
       </c>
     </row>
-    <row r="50" spans="2:4" x14ac:dyDescent="0.25">
+    <row r="50" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B50" s="2" t="s">
         <v>72</v>
       </c>
-      <c r="C50">
+      <c r="C50" s="0" t="n">
         <v>3000</v>
       </c>
       <c r="D50" s="3" t="s">
         <v>73</v>
       </c>
     </row>
-    <row r="51" spans="2:4" x14ac:dyDescent="0.25">
+    <row r="51" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B51" s="2" t="s">
         <v>74</v>
       </c>
-      <c r="C51">
+      <c r="C51" s="0" t="n">
         <v>1730</v>
       </c>
       <c r="D51" s="3" t="s">
         <v>75</v>
       </c>
     </row>
-    <row r="52" spans="2:4" x14ac:dyDescent="0.25">
+    <row r="52" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B52" s="2" t="s">
         <v>76</v>
       </c>
-      <c r="C52">
+      <c r="C52" s="0" t="n">
         <v>3000</v>
       </c>
       <c r="D52" s="3" t="s">
         <v>77</v>
       </c>
     </row>
-    <row r="53" spans="2:4" x14ac:dyDescent="0.25">
+    <row r="53" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B53" s="2" t="s">
         <v>35</v>
       </c>
-      <c r="C53">
+      <c r="C53" s="0" t="n">
         <v>-2000</v>
       </c>
       <c r="D53" s="3" t="s">
         <v>77</v>
       </c>
     </row>
-    <row r="54" spans="2:4" x14ac:dyDescent="0.25">
+    <row r="54" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B54" s="2" t="s">
         <v>78</v>
       </c>
-      <c r="C54">
+      <c r="C54" s="0" t="n">
         <v>1270</v>
       </c>
       <c r="D54" s="3" t="s">
         <v>79</v>
       </c>
     </row>
-    <row r="55" spans="2:4" x14ac:dyDescent="0.25">
+    <row r="55" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B55" s="2" t="s">
         <v>80</v>
       </c>
-      <c r="C55">
+      <c r="C55" s="0" t="n">
         <v>1190</v>
       </c>
       <c r="D55" s="3" t="s">
         <v>81</v>
       </c>
     </row>
-    <row r="56" spans="2:4" x14ac:dyDescent="0.25">
+    <row r="56" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B56" s="2" t="s">
         <v>82</v>
       </c>
-      <c r="C56">
+      <c r="C56" s="0" t="n">
         <v>1460</v>
       </c>
       <c r="D56" s="3" t="s">
         <v>83</v>
       </c>
     </row>
-    <row r="57" spans="2:4" x14ac:dyDescent="0.25">
+    <row r="57" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B57" s="2" t="s">
         <v>84</v>
       </c>
-      <c r="C57">
+      <c r="C57" s="0" t="n">
         <v>-3000</v>
       </c>
       <c r="D57" s="3" t="s">
         <v>83</v>
       </c>
     </row>
-    <row r="58" spans="2:4" x14ac:dyDescent="0.25">
+    <row r="58" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B58" s="2" t="s">
         <v>85</v>
       </c>
-      <c r="C58">
+      <c r="C58" s="0" t="n">
         <v>-700</v>
       </c>
       <c r="D58" s="3" t="s">
         <v>86</v>
       </c>
     </row>
-    <row r="59" spans="2:4" x14ac:dyDescent="0.25">
+    <row r="59" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B59" s="2" t="s">
         <v>87</v>
       </c>
-      <c r="C59">
+      <c r="C59" s="0" t="n">
         <v>3000</v>
       </c>
       <c r="D59" s="3" t="s">
         <v>88</v>
       </c>
     </row>
-    <row r="60" spans="2:4" x14ac:dyDescent="0.25">
+    <row r="60" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B60" s="2" t="s">
         <v>89</v>
       </c>
-      <c r="C60">
+      <c r="C60" s="0" t="n">
         <v>540</v>
       </c>
       <c r="D60" s="3" t="s">
         <v>90</v>
       </c>
     </row>
-    <row r="61" spans="2:4" x14ac:dyDescent="0.25">
+    <row r="61" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B61" s="2" t="s">
         <v>91</v>
       </c>
-      <c r="C61">
+      <c r="C61" s="0" t="n">
         <v>3000</v>
       </c>
       <c r="D61" s="3" t="s">
         <v>92</v>
       </c>
     </row>
-    <row r="62" spans="2:4" x14ac:dyDescent="0.25">
+    <row r="62" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B62" s="2" t="s">
         <v>93</v>
       </c>
-      <c r="C62">
+      <c r="C62" s="0" t="n">
         <v>4000</v>
       </c>
       <c r="D62" s="3" t="s">
         <v>94</v>
       </c>
     </row>
-    <row r="63" spans="2:4" x14ac:dyDescent="0.25">
+    <row r="63" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B63" s="2" t="s">
         <v>95</v>
       </c>
-      <c r="C63">
+      <c r="C63" s="0" t="n">
         <v>3000</v>
       </c>
       <c r="D63" s="3" t="s">
         <v>96</v>
       </c>
     </row>
-    <row r="64" spans="2:4" x14ac:dyDescent="0.25">
+    <row r="64" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B64" s="2" t="s">
         <v>97</v>
       </c>
-      <c r="C64">
+      <c r="C64" s="0" t="n">
         <v>3000</v>
       </c>
       <c r="D64" s="3" t="s">
         <v>98</v>
       </c>
     </row>
-    <row r="65" spans="2:4" x14ac:dyDescent="0.25">
+    <row r="65" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B65" s="2" t="s">
         <v>99</v>
       </c>
-      <c r="C65">
+      <c r="C65" s="0" t="n">
         <v>3000</v>
       </c>
       <c r="D65" s="3" t="s">
         <v>100</v>
       </c>
     </row>
-    <row r="66" spans="2:4" x14ac:dyDescent="0.25">
+    <row r="66" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B66" s="2" t="s">
         <v>101</v>
       </c>
-      <c r="C66">
+      <c r="C66" s="0" t="n">
         <v>3000</v>
       </c>
       <c r="D66" s="3" t="s">
         <v>102</v>
       </c>
     </row>
-    <row r="67" spans="2:4" x14ac:dyDescent="0.25">
+    <row r="67" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B67" s="2" t="s">
         <v>103</v>
       </c>
-      <c r="C67">
+      <c r="C67" s="0" t="n">
         <v>3000</v>
       </c>
       <c r="D67" s="3" t="s">
         <v>104</v>
       </c>
     </row>
-    <row r="68" spans="2:4" x14ac:dyDescent="0.25">
+    <row r="68" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B68" s="2" t="s">
         <v>105</v>
       </c>
-      <c r="C68">
+      <c r="C68" s="0" t="n">
         <v>3000</v>
       </c>
       <c r="D68" s="3" t="s">
         <v>106</v>
       </c>
     </row>
-    <row r="69" spans="2:4" x14ac:dyDescent="0.25">
+    <row r="69" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B69" s="2" t="s">
         <v>107</v>
       </c>
-      <c r="C69">
+      <c r="C69" s="0" t="n">
         <v>3000</v>
       </c>
       <c r="D69" s="3" t="s">
         <v>108</v>
       </c>
     </row>
-    <row r="70" spans="2:4" x14ac:dyDescent="0.25">
+    <row r="70" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B70" s="2" t="s">
         <v>109</v>
       </c>
-      <c r="C70">
+      <c r="C70" s="0" t="n">
         <v>3000</v>
       </c>
       <c r="D70" s="3" t="s">
         <v>64</v>
       </c>
     </row>
-    <row r="71" spans="2:4" x14ac:dyDescent="0.25">
+    <row r="71" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B71" s="2" t="s">
         <v>72</v>
       </c>
-      <c r="C71">
+      <c r="C71" s="0" t="n">
         <v>3000</v>
       </c>
       <c r="D71" s="3" t="s">
+        <v>110</v>
+      </c>
+    </row>
+    <row r="72" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="B72" s="2" t="s">
+        <v>76</v>
+      </c>
+      <c r="C72" s="0" t="n">
+        <v>3000</v>
+      </c>
+      <c r="D72" s="3" t="s">
         <v>111</v>
       </c>
     </row>
-    <row r="76" spans="2:4" ht="18.75" x14ac:dyDescent="0.3">
-      <c r="B76" s="4" t="s">
-        <v>110</v>
-      </c>
-      <c r="C76" s="5">
-        <f>SUM(C9:C74)</f>
-        <v>77805</v>
-      </c>
-      <c r="D76" s="3" t="s">
+    <row r="73" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="74" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="79" customFormat="false" ht="17.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="B79" s="4" t="s">
+        <v>112</v>
+      </c>
+      <c r="C79" s="5" t="n">
+        <f aca="false">SUM(C9:C77)</f>
+        <v>80805</v>
+      </c>
+      <c r="D79" s="3" t="s">
         <v>111</v>
       </c>
     </row>
-    <row r="80" spans="2:4" ht="21" x14ac:dyDescent="0.35">
-      <c r="B80" s="4"/>
-      <c r="C80" s="6"/>
-    </row>
-    <row r="151" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A151" s="2"/>
+    <row r="83" customFormat="false" ht="21" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="B83" s="4"/>
+      <c r="C83" s="6"/>
+    </row>
+    <row r="154" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A154" s="2"/>
     </row>
   </sheetData>
+  <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.511811023622047" footer="0.511811023622047"/>
-  <pageSetup orientation="portrait" horizontalDpi="300" verticalDpi="300"/>
+  <pageSetup paperSize="1" scale="100" fitToWidth="1" fitToHeight="1" pageOrder="downThenOver" orientation="portrait" blackAndWhite="false" draft="false" cellComments="none" horizontalDpi="300" verticalDpi="300" copies="1"/>
+  <headerFooter differentFirst="false" differentOddEven="false">
+    <oddHeader/>
+    <oddFooter/>
+  </headerFooter>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
tinh tien loi co yen thang 03
</commit_message>
<xml_diff>
--- a/ThuChiCoYenLinhTrung.xlsx
+++ b/ThuChiCoYenLinhTrung.xlsx
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="127" uniqueCount="113">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="129" uniqueCount="114">
   <si>
     <t xml:space="preserve">500+1100+2700-105=</t>
   </si>
@@ -356,6 +356,9 @@
   </si>
   <si>
     <t xml:space="preserve">16/03/2026</t>
+  </si>
+  <si>
+    <t xml:space="preserve">16/04/2026</t>
   </si>
   <si>
     <t xml:space="preserve">Hiện tại</t>
@@ -457,32 +460,36 @@
     <xf numFmtId="42" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
     <xf numFmtId="9" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
   </cellStyleXfs>
-  <cellXfs count="7">
+  <cellXfs count="8">
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="true" applyProtection="true">
       <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="165" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="false" applyProtection="false">
+    <xf numFmtId="165" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="165" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="165" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="true" applyProtection="true">
       <alignment horizontal="right" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="165" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
+    <xf numFmtId="165" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="4" fillId="2" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
+    <xf numFmtId="164" fontId="4" fillId="2" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
+    <xf numFmtId="164" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -738,20 +745,20 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A2:D154"/>
+  <dimension ref="A2:D155"/>
   <sheetFormatPr defaultColWidth="8.71484375" defaultRowHeight="15" customHeight="true" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="1" width="25.29"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="2" width="30.14"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="0" width="17.86"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="4" style="3" width="17.42"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="3" width="17.86"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="4" style="4" width="17.42"/>
   </cols>
   <sheetData>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B2" s="2" t="s">
         <v>0</v>
       </c>
-      <c r="C2" s="0" t="n">
+      <c r="C2" s="3" t="n">
         <f aca="false">500+1100+2700-105</f>
         <v>4195</v>
       </c>
@@ -760,7 +767,7 @@
       <c r="B9" s="2" t="s">
         <v>1</v>
       </c>
-      <c r="C9" s="0" t="n">
+      <c r="C9" s="3" t="n">
         <v>195</v>
       </c>
     </row>
@@ -768,7 +775,7 @@
       <c r="B10" s="2" t="s">
         <v>2</v>
       </c>
-      <c r="C10" s="0" t="n">
+      <c r="C10" s="3" t="n">
         <v>1836</v>
       </c>
     </row>
@@ -776,7 +783,7 @@
       <c r="B11" s="2" t="s">
         <v>3</v>
       </c>
-      <c r="C11" s="0" t="n">
+      <c r="C11" s="3" t="n">
         <v>2540</v>
       </c>
     </row>
@@ -784,10 +791,10 @@
       <c r="B12" s="2" t="s">
         <v>4</v>
       </c>
-      <c r="C12" s="0" t="n">
+      <c r="C12" s="3" t="n">
         <v>1500</v>
       </c>
-      <c r="D12" s="3" t="s">
+      <c r="D12" s="4" t="s">
         <v>5</v>
       </c>
     </row>
@@ -795,10 +802,10 @@
       <c r="B13" s="2" t="s">
         <v>6</v>
       </c>
-      <c r="C13" s="0" t="n">
-        <v>3000</v>
-      </c>
-      <c r="D13" s="3" t="s">
+      <c r="C13" s="3" t="n">
+        <v>3000</v>
+      </c>
+      <c r="D13" s="4" t="s">
         <v>7</v>
       </c>
     </row>
@@ -806,7 +813,7 @@
       <c r="B14" s="2" t="s">
         <v>8</v>
       </c>
-      <c r="C14" s="0" t="n">
+      <c r="C14" s="3" t="n">
         <v>2954</v>
       </c>
     </row>
@@ -814,10 +821,10 @@
       <c r="B15" s="2" t="s">
         <v>9</v>
       </c>
-      <c r="C15" s="0" t="n">
+      <c r="C15" s="3" t="n">
         <v>1500</v>
       </c>
-      <c r="D15" s="3" t="s">
+      <c r="D15" s="4" t="s">
         <v>10</v>
       </c>
     </row>
@@ -825,10 +832,10 @@
       <c r="B16" s="2" t="s">
         <v>11</v>
       </c>
-      <c r="C16" s="0" t="n">
-        <v>3000</v>
-      </c>
-      <c r="D16" s="3" t="s">
+      <c r="C16" s="3" t="n">
+        <v>3000</v>
+      </c>
+      <c r="D16" s="4" t="s">
         <v>12</v>
       </c>
     </row>
@@ -836,10 +843,10 @@
       <c r="B17" s="2" t="s">
         <v>13</v>
       </c>
-      <c r="C17" s="0" t="n">
+      <c r="C17" s="3" t="n">
         <v>-3000</v>
       </c>
-      <c r="D17" s="3" t="s">
+      <c r="D17" s="4" t="s">
         <v>14</v>
       </c>
     </row>
@@ -847,10 +854,10 @@
       <c r="B18" s="2" t="s">
         <v>15</v>
       </c>
-      <c r="C18" s="0" t="n">
+      <c r="C18" s="3" t="n">
         <v>1500</v>
       </c>
-      <c r="D18" s="3" t="s">
+      <c r="D18" s="4" t="s">
         <v>16</v>
       </c>
     </row>
@@ -858,10 +865,10 @@
       <c r="B19" s="2" t="s">
         <v>17</v>
       </c>
-      <c r="C19" s="0" t="n">
-        <v>3000</v>
-      </c>
-      <c r="D19" s="3" t="s">
+      <c r="C19" s="3" t="n">
+        <v>3000</v>
+      </c>
+      <c r="D19" s="4" t="s">
         <v>18</v>
       </c>
     </row>
@@ -869,10 +876,10 @@
       <c r="B20" s="2" t="s">
         <v>19</v>
       </c>
-      <c r="C20" s="0" t="n">
+      <c r="C20" s="3" t="n">
         <v>1460</v>
       </c>
-      <c r="D20" s="3" t="s">
+      <c r="D20" s="4" t="s">
         <v>20</v>
       </c>
     </row>
@@ -880,10 +887,10 @@
       <c r="B21" s="2" t="s">
         <v>21</v>
       </c>
-      <c r="C21" s="0" t="n">
+      <c r="C21" s="3" t="n">
         <v>-1000</v>
       </c>
-      <c r="D21" s="3" t="s">
+      <c r="D21" s="4" t="s">
         <v>22</v>
       </c>
     </row>
@@ -891,10 +898,10 @@
       <c r="B22" s="2" t="s">
         <v>21</v>
       </c>
-      <c r="C22" s="0" t="n">
+      <c r="C22" s="3" t="n">
         <v>-1000</v>
       </c>
-      <c r="D22" s="3" t="s">
+      <c r="D22" s="4" t="s">
         <v>23</v>
       </c>
     </row>
@@ -902,10 +909,10 @@
       <c r="B23" s="2" t="s">
         <v>24</v>
       </c>
-      <c r="C23" s="0" t="n">
+      <c r="C23" s="3" t="n">
         <v>1350</v>
       </c>
-      <c r="D23" s="3" t="s">
+      <c r="D23" s="4" t="s">
         <v>25</v>
       </c>
     </row>
@@ -913,10 +920,10 @@
       <c r="B24" s="2" t="s">
         <v>26</v>
       </c>
-      <c r="C24" s="0" t="n">
+      <c r="C24" s="3" t="n">
         <v>-600</v>
       </c>
-      <c r="D24" s="3" t="s">
+      <c r="D24" s="4" t="s">
         <v>27</v>
       </c>
     </row>
@@ -924,10 +931,10 @@
       <c r="B25" s="2" t="s">
         <v>28</v>
       </c>
-      <c r="C25" s="0" t="n">
+      <c r="C25" s="3" t="n">
         <v>-400</v>
       </c>
-      <c r="D25" s="3" t="s">
+      <c r="D25" s="4" t="s">
         <v>29</v>
       </c>
     </row>
@@ -935,10 +942,10 @@
       <c r="B26" s="2" t="s">
         <v>30</v>
       </c>
-      <c r="C26" s="0" t="n">
+      <c r="C26" s="3" t="n">
         <v>1500</v>
       </c>
-      <c r="D26" s="3" t="s">
+      <c r="D26" s="4" t="s">
         <v>29</v>
       </c>
     </row>
@@ -946,10 +953,10 @@
       <c r="B27" s="2" t="s">
         <v>31</v>
       </c>
-      <c r="C27" s="0" t="n">
+      <c r="C27" s="3" t="n">
         <v>3200</v>
       </c>
-      <c r="D27" s="3" t="s">
+      <c r="D27" s="4" t="s">
         <v>32</v>
       </c>
     </row>
@@ -957,10 +964,10 @@
       <c r="B28" s="2" t="s">
         <v>33</v>
       </c>
-      <c r="C28" s="0" t="n">
-        <v>3000</v>
-      </c>
-      <c r="D28" s="3" t="s">
+      <c r="C28" s="3" t="n">
+        <v>3000</v>
+      </c>
+      <c r="D28" s="4" t="s">
         <v>34</v>
       </c>
     </row>
@@ -968,10 +975,10 @@
       <c r="B29" s="2" t="s">
         <v>35</v>
       </c>
-      <c r="C29" s="0" t="n">
+      <c r="C29" s="3" t="n">
         <v>-2000</v>
       </c>
-      <c r="D29" s="3" t="s">
+      <c r="D29" s="4" t="s">
         <v>36</v>
       </c>
     </row>
@@ -979,10 +986,10 @@
       <c r="B30" s="2" t="s">
         <v>37</v>
       </c>
-      <c r="C30" s="0" t="n">
+      <c r="C30" s="3" t="n">
         <v>1730</v>
       </c>
-      <c r="D30" s="3" t="s">
+      <c r="D30" s="4" t="s">
         <v>38</v>
       </c>
     </row>
@@ -990,10 +997,10 @@
       <c r="B31" s="2" t="s">
         <v>39</v>
       </c>
-      <c r="C31" s="0" t="n">
+      <c r="C31" s="3" t="n">
         <v>-1000</v>
       </c>
-      <c r="D31" s="3" t="s">
+      <c r="D31" s="4" t="s">
         <v>38</v>
       </c>
     </row>
@@ -1001,10 +1008,10 @@
       <c r="B32" s="2" t="s">
         <v>40</v>
       </c>
-      <c r="C32" s="0" t="n">
+      <c r="C32" s="3" t="n">
         <v>1500</v>
       </c>
-      <c r="D32" s="3" t="s">
+      <c r="D32" s="4" t="s">
         <v>41</v>
       </c>
     </row>
@@ -1012,10 +1019,10 @@
       <c r="B33" s="2" t="s">
         <v>42</v>
       </c>
-      <c r="C33" s="0" t="n">
+      <c r="C33" s="3" t="n">
         <v>2000</v>
       </c>
-      <c r="D33" s="3" t="s">
+      <c r="D33" s="4" t="s">
         <v>43</v>
       </c>
     </row>
@@ -1023,10 +1030,10 @@
       <c r="B34" s="2" t="s">
         <v>44</v>
       </c>
-      <c r="C34" s="0" t="n">
-        <v>3000</v>
-      </c>
-      <c r="D34" s="3" t="s">
+      <c r="C34" s="3" t="n">
+        <v>3000</v>
+      </c>
+      <c r="D34" s="4" t="s">
         <v>45</v>
       </c>
     </row>
@@ -1034,10 +1041,10 @@
       <c r="B35" s="2" t="s">
         <v>46</v>
       </c>
-      <c r="C35" s="0" t="n">
+      <c r="C35" s="3" t="n">
         <v>2000</v>
       </c>
-      <c r="D35" s="3" t="s">
+      <c r="D35" s="4" t="s">
         <v>47</v>
       </c>
     </row>
@@ -1045,10 +1052,10 @@
       <c r="B36" s="2" t="s">
         <v>48</v>
       </c>
-      <c r="C36" s="0" t="n">
+      <c r="C36" s="3" t="n">
         <v>2930</v>
       </c>
-      <c r="D36" s="3" t="s">
+      <c r="D36" s="4" t="s">
         <v>49</v>
       </c>
     </row>
@@ -1056,10 +1063,10 @@
       <c r="B37" s="2" t="s">
         <v>50</v>
       </c>
-      <c r="C37" s="0" t="n">
+      <c r="C37" s="3" t="n">
         <v>-3000</v>
       </c>
-      <c r="D37" s="3" t="s">
+      <c r="D37" s="4" t="s">
         <v>51</v>
       </c>
     </row>
@@ -1067,10 +1074,10 @@
       <c r="B38" s="2" t="s">
         <v>44</v>
       </c>
-      <c r="C38" s="0" t="n">
-        <v>3000</v>
-      </c>
-      <c r="D38" s="3" t="s">
+      <c r="C38" s="3" t="n">
+        <v>3000</v>
+      </c>
+      <c r="D38" s="4" t="s">
         <v>52</v>
       </c>
     </row>
@@ -1078,10 +1085,10 @@
       <c r="B39" s="2" t="s">
         <v>53</v>
       </c>
-      <c r="C39" s="0" t="n">
+      <c r="C39" s="3" t="n">
         <v>1730</v>
       </c>
-      <c r="D39" s="3" t="s">
+      <c r="D39" s="4" t="s">
         <v>54</v>
       </c>
     </row>
@@ -1089,10 +1096,10 @@
       <c r="B40" s="2" t="s">
         <v>55</v>
       </c>
-      <c r="C40" s="0" t="n">
+      <c r="C40" s="3" t="n">
         <v>-2000</v>
       </c>
-      <c r="D40" s="3" t="s">
+      <c r="D40" s="4" t="s">
         <v>56</v>
       </c>
     </row>
@@ -1100,10 +1107,10 @@
       <c r="B41" s="2" t="s">
         <v>57</v>
       </c>
-      <c r="C41" s="0" t="n">
+      <c r="C41" s="3" t="n">
         <v>1920</v>
       </c>
-      <c r="D41" s="3" t="s">
+      <c r="D41" s="4" t="s">
         <v>58</v>
       </c>
     </row>
@@ -1111,10 +1118,10 @@
       <c r="B42" s="2" t="s">
         <v>35</v>
       </c>
-      <c r="C42" s="0" t="n">
+      <c r="C42" s="3" t="n">
         <v>-2000</v>
       </c>
-      <c r="D42" s="3" t="s">
+      <c r="D42" s="4" t="s">
         <v>59</v>
       </c>
     </row>
@@ -1122,10 +1129,10 @@
       <c r="B43" s="2" t="s">
         <v>60</v>
       </c>
-      <c r="C43" s="0" t="n">
+      <c r="C43" s="3" t="n">
         <v>1730</v>
       </c>
-      <c r="D43" s="3" t="s">
+      <c r="D43" s="4" t="s">
         <v>61</v>
       </c>
     </row>
@@ -1133,10 +1140,10 @@
       <c r="B44" s="2" t="s">
         <v>35</v>
       </c>
-      <c r="C44" s="0" t="n">
+      <c r="C44" s="3" t="n">
         <v>-2000</v>
       </c>
-      <c r="D44" s="3" t="s">
+      <c r="D44" s="4" t="s">
         <v>62</v>
       </c>
     </row>
@@ -1144,10 +1151,10 @@
       <c r="B45" s="2" t="s">
         <v>63</v>
       </c>
-      <c r="C45" s="0" t="n">
-        <v>3000</v>
-      </c>
-      <c r="D45" s="3" t="s">
+      <c r="C45" s="3" t="n">
+        <v>3000</v>
+      </c>
+      <c r="D45" s="4" t="s">
         <v>64</v>
       </c>
     </row>
@@ -1155,10 +1162,10 @@
       <c r="B46" s="2" t="s">
         <v>65</v>
       </c>
-      <c r="C46" s="0" t="n">
+      <c r="C46" s="3" t="n">
         <v>810</v>
       </c>
-      <c r="D46" s="3" t="s">
+      <c r="D46" s="4" t="s">
         <v>64</v>
       </c>
     </row>
@@ -1166,10 +1173,10 @@
       <c r="B47" s="2" t="s">
         <v>66</v>
       </c>
-      <c r="C47" s="0" t="n">
+      <c r="C47" s="3" t="n">
         <v>-3000</v>
       </c>
-      <c r="D47" s="3" t="s">
+      <c r="D47" s="4" t="s">
         <v>67</v>
       </c>
     </row>
@@ -1177,10 +1184,10 @@
       <c r="B48" s="2" t="s">
         <v>68</v>
       </c>
-      <c r="C48" s="0" t="n">
+      <c r="C48" s="3" t="n">
         <v>3430</v>
       </c>
-      <c r="D48" s="3" t="s">
+      <c r="D48" s="4" t="s">
         <v>69</v>
       </c>
     </row>
@@ -1188,10 +1195,10 @@
       <c r="B49" s="2" t="s">
         <v>70</v>
       </c>
-      <c r="C49" s="0" t="n">
+      <c r="C49" s="3" t="n">
         <v>-5000</v>
       </c>
-      <c r="D49" s="3" t="s">
+      <c r="D49" s="4" t="s">
         <v>71</v>
       </c>
     </row>
@@ -1199,10 +1206,10 @@
       <c r="B50" s="2" t="s">
         <v>72</v>
       </c>
-      <c r="C50" s="0" t="n">
-        <v>3000</v>
-      </c>
-      <c r="D50" s="3" t="s">
+      <c r="C50" s="3" t="n">
+        <v>3000</v>
+      </c>
+      <c r="D50" s="4" t="s">
         <v>73</v>
       </c>
     </row>
@@ -1210,10 +1217,10 @@
       <c r="B51" s="2" t="s">
         <v>74</v>
       </c>
-      <c r="C51" s="0" t="n">
+      <c r="C51" s="3" t="n">
         <v>1730</v>
       </c>
-      <c r="D51" s="3" t="s">
+      <c r="D51" s="4" t="s">
         <v>75</v>
       </c>
     </row>
@@ -1221,10 +1228,10 @@
       <c r="B52" s="2" t="s">
         <v>76</v>
       </c>
-      <c r="C52" s="0" t="n">
-        <v>3000</v>
-      </c>
-      <c r="D52" s="3" t="s">
+      <c r="C52" s="3" t="n">
+        <v>3000</v>
+      </c>
+      <c r="D52" s="4" t="s">
         <v>77</v>
       </c>
     </row>
@@ -1232,10 +1239,10 @@
       <c r="B53" s="2" t="s">
         <v>35</v>
       </c>
-      <c r="C53" s="0" t="n">
+      <c r="C53" s="3" t="n">
         <v>-2000</v>
       </c>
-      <c r="D53" s="3" t="s">
+      <c r="D53" s="4" t="s">
         <v>77</v>
       </c>
     </row>
@@ -1243,10 +1250,10 @@
       <c r="B54" s="2" t="s">
         <v>78</v>
       </c>
-      <c r="C54" s="0" t="n">
+      <c r="C54" s="3" t="n">
         <v>1270</v>
       </c>
-      <c r="D54" s="3" t="s">
+      <c r="D54" s="4" t="s">
         <v>79</v>
       </c>
     </row>
@@ -1254,10 +1261,10 @@
       <c r="B55" s="2" t="s">
         <v>80</v>
       </c>
-      <c r="C55" s="0" t="n">
+      <c r="C55" s="3" t="n">
         <v>1190</v>
       </c>
-      <c r="D55" s="3" t="s">
+      <c r="D55" s="4" t="s">
         <v>81</v>
       </c>
     </row>
@@ -1265,10 +1272,10 @@
       <c r="B56" s="2" t="s">
         <v>82</v>
       </c>
-      <c r="C56" s="0" t="n">
+      <c r="C56" s="3" t="n">
         <v>1460</v>
       </c>
-      <c r="D56" s="3" t="s">
+      <c r="D56" s="4" t="s">
         <v>83</v>
       </c>
     </row>
@@ -1276,10 +1283,10 @@
       <c r="B57" s="2" t="s">
         <v>84</v>
       </c>
-      <c r="C57" s="0" t="n">
+      <c r="C57" s="3" t="n">
         <v>-3000</v>
       </c>
-      <c r="D57" s="3" t="s">
+      <c r="D57" s="4" t="s">
         <v>83</v>
       </c>
     </row>
@@ -1287,10 +1294,10 @@
       <c r="B58" s="2" t="s">
         <v>85</v>
       </c>
-      <c r="C58" s="0" t="n">
+      <c r="C58" s="3" t="n">
         <v>-700</v>
       </c>
-      <c r="D58" s="3" t="s">
+      <c r="D58" s="4" t="s">
         <v>86</v>
       </c>
     </row>
@@ -1298,10 +1305,10 @@
       <c r="B59" s="2" t="s">
         <v>87</v>
       </c>
-      <c r="C59" s="0" t="n">
-        <v>3000</v>
-      </c>
-      <c r="D59" s="3" t="s">
+      <c r="C59" s="3" t="n">
+        <v>3000</v>
+      </c>
+      <c r="D59" s="4" t="s">
         <v>88</v>
       </c>
     </row>
@@ -1309,10 +1316,10 @@
       <c r="B60" s="2" t="s">
         <v>89</v>
       </c>
-      <c r="C60" s="0" t="n">
+      <c r="C60" s="3" t="n">
         <v>540</v>
       </c>
-      <c r="D60" s="3" t="s">
+      <c r="D60" s="4" t="s">
         <v>90</v>
       </c>
     </row>
@@ -1320,10 +1327,10 @@
       <c r="B61" s="2" t="s">
         <v>91</v>
       </c>
-      <c r="C61" s="0" t="n">
-        <v>3000</v>
-      </c>
-      <c r="D61" s="3" t="s">
+      <c r="C61" s="3" t="n">
+        <v>3000</v>
+      </c>
+      <c r="D61" s="4" t="s">
         <v>92</v>
       </c>
     </row>
@@ -1331,10 +1338,10 @@
       <c r="B62" s="2" t="s">
         <v>93</v>
       </c>
-      <c r="C62" s="0" t="n">
+      <c r="C62" s="3" t="n">
         <v>4000</v>
       </c>
-      <c r="D62" s="3" t="s">
+      <c r="D62" s="4" t="s">
         <v>94</v>
       </c>
     </row>
@@ -1342,10 +1349,10 @@
       <c r="B63" s="2" t="s">
         <v>95</v>
       </c>
-      <c r="C63" s="0" t="n">
-        <v>3000</v>
-      </c>
-      <c r="D63" s="3" t="s">
+      <c r="C63" s="3" t="n">
+        <v>3000</v>
+      </c>
+      <c r="D63" s="4" t="s">
         <v>96</v>
       </c>
     </row>
@@ -1353,10 +1360,10 @@
       <c r="B64" s="2" t="s">
         <v>97</v>
       </c>
-      <c r="C64" s="0" t="n">
-        <v>3000</v>
-      </c>
-      <c r="D64" s="3" t="s">
+      <c r="C64" s="3" t="n">
+        <v>3000</v>
+      </c>
+      <c r="D64" s="4" t="s">
         <v>98</v>
       </c>
     </row>
@@ -1364,10 +1371,10 @@
       <c r="B65" s="2" t="s">
         <v>99</v>
       </c>
-      <c r="C65" s="0" t="n">
-        <v>3000</v>
-      </c>
-      <c r="D65" s="3" t="s">
+      <c r="C65" s="3" t="n">
+        <v>3000</v>
+      </c>
+      <c r="D65" s="4" t="s">
         <v>100</v>
       </c>
     </row>
@@ -1375,10 +1382,10 @@
       <c r="B66" s="2" t="s">
         <v>101</v>
       </c>
-      <c r="C66" s="0" t="n">
-        <v>3000</v>
-      </c>
-      <c r="D66" s="3" t="s">
+      <c r="C66" s="3" t="n">
+        <v>3000</v>
+      </c>
+      <c r="D66" s="4" t="s">
         <v>102</v>
       </c>
     </row>
@@ -1386,10 +1393,10 @@
       <c r="B67" s="2" t="s">
         <v>103</v>
       </c>
-      <c r="C67" s="0" t="n">
-        <v>3000</v>
-      </c>
-      <c r="D67" s="3" t="s">
+      <c r="C67" s="3" t="n">
+        <v>3000</v>
+      </c>
+      <c r="D67" s="4" t="s">
         <v>104</v>
       </c>
     </row>
@@ -1397,10 +1404,10 @@
       <c r="B68" s="2" t="s">
         <v>105</v>
       </c>
-      <c r="C68" s="0" t="n">
-        <v>3000</v>
-      </c>
-      <c r="D68" s="3" t="s">
+      <c r="C68" s="3" t="n">
+        <v>3000</v>
+      </c>
+      <c r="D68" s="4" t="s">
         <v>106</v>
       </c>
     </row>
@@ -1408,10 +1415,10 @@
       <c r="B69" s="2" t="s">
         <v>107</v>
       </c>
-      <c r="C69" s="0" t="n">
-        <v>3000</v>
-      </c>
-      <c r="D69" s="3" t="s">
+      <c r="C69" s="3" t="n">
+        <v>3000</v>
+      </c>
+      <c r="D69" s="4" t="s">
         <v>108</v>
       </c>
     </row>
@@ -1419,10 +1426,10 @@
       <c r="B70" s="2" t="s">
         <v>109</v>
       </c>
-      <c r="C70" s="0" t="n">
-        <v>3000</v>
-      </c>
-      <c r="D70" s="3" t="s">
+      <c r="C70" s="3" t="n">
+        <v>3000</v>
+      </c>
+      <c r="D70" s="4" t="s">
         <v>64</v>
       </c>
     </row>
@@ -1430,10 +1437,10 @@
       <c r="B71" s="2" t="s">
         <v>72</v>
       </c>
-      <c r="C71" s="0" t="n">
-        <v>3000</v>
-      </c>
-      <c r="D71" s="3" t="s">
+      <c r="C71" s="3" t="n">
+        <v>3000</v>
+      </c>
+      <c r="D71" s="4" t="s">
         <v>110</v>
       </c>
     </row>
@@ -1441,33 +1448,44 @@
       <c r="B72" s="2" t="s">
         <v>76</v>
       </c>
-      <c r="C72" s="0" t="n">
-        <v>3000</v>
-      </c>
-      <c r="D72" s="3" t="s">
+      <c r="C72" s="3" t="n">
+        <v>3000</v>
+      </c>
+      <c r="D72" s="4" t="s">
         <v>111</v>
       </c>
     </row>
-    <row r="73" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="73" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="B73" s="2" t="s">
+        <v>87</v>
+      </c>
+      <c r="C73" s="3" t="n">
+        <v>3000</v>
+      </c>
+      <c r="D73" s="4" t="s">
+        <v>112</v>
+      </c>
+    </row>
     <row r="74" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
-    <row r="79" customFormat="false" ht="17.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B79" s="4" t="s">
+    <row r="75" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="80" customFormat="false" ht="17.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="B80" s="5" t="s">
+        <v>113</v>
+      </c>
+      <c r="C80" s="6" t="n">
+        <f aca="false">SUM(C9:C78)</f>
+        <v>83805</v>
+      </c>
+      <c r="D80" s="4" t="s">
         <v>112</v>
       </c>
-      <c r="C79" s="5" t="n">
-        <f aca="false">SUM(C9:C77)</f>
-        <v>80805</v>
-      </c>
-      <c r="D79" s="3" t="s">
-        <v>111</v>
-      </c>
-    </row>
-    <row r="83" customFormat="false" ht="21" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B83" s="4"/>
-      <c r="C83" s="6"/>
-    </row>
-    <row r="154" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A154" s="2"/>
+    </row>
+    <row r="84" customFormat="false" ht="21" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="B84" s="5"/>
+      <c r="C84" s="7"/>
+    </row>
+    <row r="155" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A155" s="2"/>
     </row>
   </sheetData>
   <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>

</xml_diff>

<commit_message>
duy tinh tien loi thang 04
</commit_message>
<xml_diff>
--- a/ThuChiCoYenLinhTrung.xlsx
+++ b/ThuChiCoYenLinhTrung.xlsx
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="129" uniqueCount="114">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="131" uniqueCount="115">
   <si>
     <t xml:space="preserve">500+1100+2700-105=</t>
   </si>
@@ -359,6 +359,9 @@
   </si>
   <si>
     <t xml:space="preserve">16/04/2026</t>
+  </si>
+  <si>
+    <t xml:space="preserve">16/05/2026</t>
   </si>
   <si>
     <t xml:space="preserve">Hiện tại</t>
@@ -745,7 +748,7 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A2:D155"/>
+  <dimension ref="A2:D156"/>
   <sheetFormatPr defaultColWidth="8.71484375" defaultRowHeight="15" customHeight="true" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="1" width="25.29"/>
@@ -1466,26 +1469,37 @@
         <v>112</v>
       </c>
     </row>
-    <row r="74" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="74" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="B74" s="2" t="s">
+        <v>91</v>
+      </c>
+      <c r="C74" s="3" t="n">
+        <v>3000</v>
+      </c>
+      <c r="D74" s="4" t="s">
+        <v>113</v>
+      </c>
+    </row>
     <row r="75" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
-    <row r="80" customFormat="false" ht="17.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B80" s="5" t="s">
+    <row r="76" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="81" customFormat="false" ht="17.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="B81" s="5" t="s">
+        <v>114</v>
+      </c>
+      <c r="C81" s="6" t="n">
+        <f aca="false">SUM(C9:C79)</f>
+        <v>86805</v>
+      </c>
+      <c r="D81" s="4" t="s">
         <v>113</v>
       </c>
-      <c r="C80" s="6" t="n">
-        <f aca="false">SUM(C9:C78)</f>
-        <v>83805</v>
-      </c>
-      <c r="D80" s="4" t="s">
-        <v>112</v>
-      </c>
-    </row>
-    <row r="84" customFormat="false" ht="21" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B84" s="5"/>
-      <c r="C84" s="7"/>
-    </row>
-    <row r="155" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A155" s="2"/>
+    </row>
+    <row r="85" customFormat="false" ht="21" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="B85" s="5"/>
+      <c r="C85" s="7"/>
+    </row>
+    <row r="156" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A156" s="2"/>
     </row>
   </sheetData>
   <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>

</xml_diff>